<commit_message>
Bridge PCB3: add 0Ω bypass jumper for 5V regulator
Allows future conversion to a 5V power source by removing the
regulator and changing only the LED current-limiting resistor
values, instead of requiring a board respin.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/enterprise documentation/PCB Design/BOM_BridgePCB3.xlsx
+++ b/enterprise documentation/PCB Design/BOM_BridgePCB3.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Saucer PCB 3_PCB 3_2026-05-" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Saucer PCB 3_PCB 3_2026-08-" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="71">
   <si>
     <t>No.</t>
   </si>
@@ -184,6 +184,21 @@
     <t>8</t>
   </si>
   <si>
+    <t>0Ω</t>
+  </si>
+  <si>
+    <t>R213</t>
+  </si>
+  <si>
+    <t>0603WAF0000T5E</t>
+  </si>
+  <si>
+    <t>C21189</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
     <t>DY-SV17F 4</t>
   </si>
   <si>
@@ -193,7 +208,7 @@
     <t>DY-SV17F</t>
   </si>
   <si>
-    <t>9</t>
+    <t>10</t>
   </si>
   <si>
     <t>LM1117S-5.0(MS)</t>
@@ -585,7 +600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -861,58 +876,90 @@
         <v>58</v>
       </c>
       <c r="E9" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" t="s">
         <v>59</v>
       </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>14</v>
-      </c>
       <c r="H9" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="I9" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="J9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
         <v>14</v>
       </c>
       <c r="G10" t="s">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>14</v>
       </c>
       <c r="I10" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>65</v>
       </c>
-      <c r="J10" t="s">
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" t="s">
+        <v>70</v>
+      </c>
+      <c r="J11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>